<commit_message>
feat: monitor licitaciones - selector dias, endpoint datos, limpieza archivos viejos
</commit_message>
<xml_diff>
--- a/data/2026-02/flujo_licitaciones_2026-02-24.xlsx
+++ b/data/2026-02/flujo_licitaciones_2026-02-24.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔗 Flujo Cruzado" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⚠️ Alertas Riesgo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⏳ Licitaciones Abiertas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,102 +430,102 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>fecha</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>organismo_contratante</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>tipo_proceso_bora</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>link_bora</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>proveedor_adjudicado</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>cuit_proveedor</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>monto_adjudicado_bora</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>en_comprar</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>procesos_comprar</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>unidad_comprar</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>nro_proceso_comprar</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>cobro_en_tgn</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>beneficiario_tgn</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>monto_cobrado_tgn</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>etapa</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>alerta</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>indicadores_riesgo</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>score_riesgo_licit</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>indice_riesgo_licit</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>nivel_riesgo_licit</t>
         </is>
@@ -572,14 +584,14 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>🟡 Adjudicación mismo día de publicación</t>
+          <t>✅ Sin alertas</t>
         </is>
       </c>
       <c r="R2" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>1.36</v>
+        <v>0</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -648,18 +660,18 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>🔴 Contratación Directa | 🟡 Adjudicación mismo día de publicación</t>
+          <t>🔴 Contratación Directa</t>
         </is>
       </c>
       <c r="R3" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="S3" t="n">
-        <v>4.09</v>
+        <v>2.73</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Medio</t>
+          <t>Bajo</t>
         </is>
       </c>
     </row>
@@ -716,14 +728,14 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>🟡 Adjudicación mismo día de publicación</t>
+          <t>✅ Sin alertas</t>
         </is>
       </c>
       <c r="R4" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>1.36</v>
+        <v>0</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
@@ -784,14 +796,14 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>🟡 Adjudicación mismo día de publicación</t>
+          <t>✅ Sin alertas</t>
         </is>
       </c>
       <c r="R5" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>1.36</v>
+        <v>0</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -848,14 +860,14 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>🟡 Adjudicación mismo día de publicación</t>
+          <t>✅ Sin alertas</t>
         </is>
       </c>
       <c r="R6" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>1.36</v>
+        <v>0</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -916,14 +928,14 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>🟡 Adjudicación mismo día de publicación</t>
+          <t>✅ Sin alertas</t>
         </is>
       </c>
       <c r="R7" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>1.36</v>
+        <v>0</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -942,108 +954,53 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>fecha</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>organismo_contratante</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>tipo_proceso_bora</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>link_bora</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>proveedor_adjudicado</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>cuit_proveedor</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>monto_adjudicado_bora</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>en_comprar</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>procesos_comprar</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>unidad_comprar</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>nro_proceso_comprar</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>cobro_en_tgn</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>beneficiario_tgn</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>monto_cobrado_tgn</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>etapa</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>alerta</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>indicadores_riesgo</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>score_riesgo_licit</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>indice_riesgo_licit</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>nivel_riesgo_licit</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>fecha_extraccion</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>nro_proceso</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>nombre_proceso</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>tipo_proceso</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>fecha_apertura</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>estado</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>unidad_ejecutora</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>fuente</t>
         </is>
       </c>
     </row>
@@ -1055,71 +1012,559 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AGENCIA DE RECAUDACIÓN Y CONTROL ADUANERO - DIRECCIÓN REGIONAL ADUANERA CUYO</t>
+          <t>84/71-0020-LPR26</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Contratación Directa 01/26</t>
+          <t>CONTRATACIÓN DE SERVICIO DE FUMIGACIÓN, DESRATIZACIÓN Y CONTROL DE PLAGAS CON OPCIÓN APRORROGA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.boletinoficial.gob.ar/detalleAviso/tercera/2408003/20260224</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ELEVADORES  EXON  S.A.S</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>25/02/2026 08:00 Hrs.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Publicado</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>$1.176.000,00</t>
+          <t>84/71 - Liceo Militar General Roca</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>❌ NO</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>❌ NO</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>⚠️ SIN CUIT EXTRAÍDO</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>📋 SOLO BORA</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>🔴 Contratación Directa | 🟡 Adjudicación mismo día de publicación</t>
-        </is>
-      </c>
-      <c r="R2" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="S2" t="n">
-        <v>4.09</v>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>https://comprar.gob.ar/Compras.aspx?qs=W1HXHGHtH10=</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Comprar.gob.ar</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>40/16-0047-CDI26</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CALIBRACIÓN ANUAL DE TALLER DE HÉLICES</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>25/02/2026 08:00 Hrs.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Publicado</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>40/016 - AREA MATERIAL QUILMES</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://comprar.gob.ar/Compras.aspx?qs=W1HXHGHtH10=</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Comprar.gob.ar</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>40/16-0038-CDI26</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Adquisición de utensillos y menaje</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>25/02/2026 08:00 Hrs.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Publicado</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>40/016 - AREA MATERIAL QUILMES</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://comprar.gob.ar/Compras.aspx?qs=W1HXHGHtH10=</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Comprar.gob.ar</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>74/45-0032-LPR26</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ADQUISICION DE BINOCULARES PARA EL PN ISLAS DE SANTA FE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Licitación Privada</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>25/02/2026 08:00 Hrs.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Publicado</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>74/45 - Parque Nacional Islas de Santa Fe</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://comprar.gob.ar/Compras.aspx?qs=W1HXHGHtH10=</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Comprar.gob.ar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>40/16-0031-CDI26</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ADQUISICIÓN DE BATERIAS RECARGABLES</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>25/02/2026 08:00 Hrs.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Publicado</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>40/016 - AREA MATERIAL QUILMES</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://comprar.gob.ar/Compras.aspx?qs=W1HXHGHtH10=</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Comprar.gob.ar</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>340/1-0001-CDI26</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SERVICIO DE RECARGA DE MATAFUEGOS FIJOS Y VEHICULARES  - SSPOYSLD</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>25/02/2026 09:00 Hrs.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Publicado</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>340/001 - Dirección General de Administración - SSSLD</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://comprar.gob.ar/Compras.aspx?qs=W1HXHGHtH10=</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Comprar.gob.ar</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>84/26-1236-LPU25</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Reparación de Endoscopios del Servicio de Gastroenterología del HMC</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>25/02/2026 09:00 Hrs.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Publicado</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>84/26 - Hospital Militar Central 601</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://comprar.gob.ar/Compras.aspx?qs=W1HXHGHtH10=</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Comprar.gob.ar</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>84/135-0138-LPR26</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ADQUISICIÓN DE UN SERVICIO INTEGRAL DE MANT. PREVENTIVO Y CORRECTIVO DE DOS (2) ASCENSORES DE LA DGM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Licitación Privada</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>25/02/2026 09:00 Hrs.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Publicado</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>84/135 - Dirección General de Material</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://comprar.gob.ar/Compras.aspx?qs=W1HXHGHtH10=</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Comprar.gob.ar</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>40/19-0090-CDI26</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ADQUISICION DE HIPOCLORITO DE SODIO</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>25/02/2026 09:00 Hrs.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Publicado</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>40/019 - UOC  RTA</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://comprar.gob.ar/Compras.aspx?qs=W1HXHGHtH10=</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Comprar.gob.ar</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>40/24-0027-CDI26</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>“Servicio de mantenimiento de la Red Wan – G2 (Segundo Llamado)”</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>25/02/2026 09:00 Hrs.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Publicado</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>40/024 - UOC CRV</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://comprar.gob.ar/Compras.aspx?qs=W1HXHGHtH10=</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Comprar.gob.ar</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>12345678910...</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://comprar.gob.ar/Compras.aspx?qs=W1HXHGHtH10=</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Comprar.gob.ar</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://comprar.gob.ar/Compras.aspx?qs=W1HXHGHtH10=</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Comprar.gob.ar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mi actualizacion para Railway
</commit_message>
<xml_diff>
--- a/data/2026-02/flujo_licitaciones_2026-02-24.xlsx
+++ b/data/2026-02/flujo_licitaciones_2026-02-24.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔗 Flujo Cruzado" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⏳ Licitaciones Abiertas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⚠️ Alertas Riesgo" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -584,14 +585,14 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>✅ Sin alertas</t>
+          <t>🟡 Adjudicación mismo día de publicación</t>
         </is>
       </c>
       <c r="R2" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="S2" t="n">
-        <v>0</v>
+        <v>1.36</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -660,18 +661,18 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>🔴 Contratación Directa</t>
+          <t>🔴 Contratación Directa | 🟡 Adjudicación mismo día de publicación</t>
         </is>
       </c>
       <c r="R3" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="S3" t="n">
-        <v>2.73</v>
+        <v>4.09</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Bajo</t>
+          <t>Medio</t>
         </is>
       </c>
     </row>
@@ -728,14 +729,14 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>✅ Sin alertas</t>
+          <t>🟡 Adjudicación mismo día de publicación</t>
         </is>
       </c>
       <c r="R4" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="S4" t="n">
-        <v>0</v>
+        <v>1.36</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
@@ -796,14 +797,14 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>✅ Sin alertas</t>
+          <t>🟡 Adjudicación mismo día de publicación</t>
         </is>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="S5" t="n">
-        <v>0</v>
+        <v>1.36</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -860,14 +861,14 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>✅ Sin alertas</t>
+          <t>🟡 Adjudicación mismo día de publicación</t>
         </is>
       </c>
       <c r="R6" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="S6" t="n">
-        <v>0</v>
+        <v>1.36</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -928,14 +929,14 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>✅ Sin alertas</t>
+          <t>🟡 Adjudicación mismo día de publicación</t>
         </is>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
+        <v>1.36</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -1571,4 +1572,196 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>organismo_contratante</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>tipo_proceso_bora</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>link_bora</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>proveedor_adjudicado</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>cuit_proveedor</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>monto_adjudicado_bora</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>en_comprar</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>procesos_comprar</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>unidad_comprar</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>nro_proceso_comprar</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>cobro_en_tgn</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>beneficiario_tgn</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>monto_cobrado_tgn</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>etapa</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>alerta</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>indicadores_riesgo</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>score_riesgo_licit</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>indice_riesgo_licit</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>nivel_riesgo_licit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AGENCIA DE RECAUDACIÓN Y CONTROL ADUANERO - DIRECCIÓN REGIONAL ADUANERA CUYO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Contratación Directa 01/26</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://www.boletinoficial.gob.ar/detalleAviso/tercera/2408003/20260224</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ELEVADORES  EXON  S.A.S</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>$1.176.000,00</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>❌ NO</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>❌ NO</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>⚠️ SIN CUIT EXTRAÍDO</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>📋 SOLO BORA</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>🔴 Contratación Directa | 🟡 Adjudicación mismo día de publicación</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="S2" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>